<commit_message>
Made changes Slovakia, USA and Romania Bproces and many page level changes
</commit_message>
<xml_diff>
--- a/Data/testDataUS.xlsx
+++ b/Data/testDataUS.xlsx
@@ -178,10 +178,10 @@
     <t>Mr</t>
   </si>
   <si>
-    <t>Soledad</t>
-  </si>
-  <si>
-    <t>Lowe</t>
+    <t>Davion</t>
+  </si>
+  <si>
+    <t>Upton</t>
   </si>
   <si>
     <t>(202) 555-0147</t>
@@ -268,10 +268,10 @@
     <t>USA Pay Group</t>
   </si>
   <si>
-    <t>{"name":"TimeoutError"}</t>
-  </si>
-  <si>
-    <t>Failed</t>
+    <t>10651502</t>
+  </si>
+  <si>
+    <t>Passed</t>
   </si>
 </sst>
 </file>
@@ -348,7 +348,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="J2" s="13">
         <f>TODAY()-31</f>
-        <v>45552</v>
+        <v>45556</v>
       </c>
       <c r="K2" s="8" t="s">
         <v>52</v>
@@ -1068,11 +1068,11 @@
       </c>
       <c r="V2" s="18">
         <f>J2</f>
-        <v>45552</v>
+        <v>45556</v>
       </c>
       <c r="W2" s="13">
         <f>TODAY()+20</f>
-        <v>45603</v>
+        <v>45607</v>
       </c>
       <c r="X2" s="19" t="s">
         <v>64</v>
@@ -1130,13 +1130,13 @@
       </c>
       <c r="AP2" s="26">
         <f t="array" ref="AP2">_xlfn.RANDARRAY(1,1,123456789,999999999,FALSE)</f>
-        <v>601816286.1566352</v>
+        <v>156895655.41836035</v>
       </c>
       <c r="AQ2" s="21" t="s">
         <v>78</v>
       </c>
       <c r="AR2" s="27">
-        <v>35591</v>
+        <v>35226</v>
       </c>
       <c r="AS2" s="8" t="s">
         <v>52</v>

</xml_diff>

<commit_message>
Latest changes on the Job Transfer,to handle with and with out manager Appproval
</commit_message>
<xml_diff>
--- a/Data/testDataUS.xlsx
+++ b/Data/testDataUS.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E7CA077-16A1-4621-961C-3C11F222CB64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E498E69-0093-4108-857D-DB6D0360D88E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1025,7 +1025,7 @@
       </c>
       <c r="J2" s="13">
         <f ca="1">TODAY()-31</f>
-        <v>45549</v>
+        <v>45564</v>
       </c>
       <c r="K2" s="8" t="s">
         <v>52</v>
@@ -1062,11 +1062,11 @@
       </c>
       <c r="V2" s="18">
         <f ca="1">J2</f>
-        <v>45549</v>
+        <v>45564</v>
       </c>
       <c r="W2" s="13">
         <f ca="1">TODAY()+20</f>
-        <v>45600</v>
+        <v>45615</v>
       </c>
       <c r="X2" s="19" t="s">
         <v>64</v>

</xml_diff>